<commit_message>
실제 검사시간(Result_Time_Data.csv) 반영해 Tact_sec 채움
Run Id별 Finish−Start를 실제 검사시간으로 계산해 DOE 엑셀 Tact_sec 갱신
(기존 이미지 타임스탬프 근사 → 작업 전체 소요시간으로 대체).

- 실험데이터/Result_Time_Data.csv 업로드
- 38런 Tact_sec 채움(D26-04는 2런 3708/3712 평균), Recipe Id로 매칭
- Word 보고서 §4에 Result_Time_Data.csv 추가, §5 Tact_sec 출처 정정

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEDPo1aa2m4Ui6JuqiXEbY
</commit_message>
<xml_diff>
--- a/실험데이터/공정모델링_DOE_2anchor_3anchor_Fmin32_측정직경모델/공정모델링_DOE_2anchor_3anchor_Fmin32_측정직경모델.xlsx
+++ b/실험데이터/공정모델링_DOE_2anchor_3anchor_Fmin32_측정직경모델/공정모델링_DOE_2anchor_3anchor_Fmin32_측정직경모델.xlsx
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="AG2" s="4" t="n">
-        <v>60</v>
+        <v>169</v>
       </c>
       <c r="AH2" s="4" t="n"/>
       <c r="AI2" t="inlineStr">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="AG3" s="4" t="n">
-        <v>60</v>
+        <v>154</v>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" t="inlineStr">
@@ -1576,7 +1576,7 @@
         </is>
       </c>
       <c r="AG4" s="4" t="n">
-        <v>58</v>
+        <v>149</v>
       </c>
       <c r="AH4" s="4" t="n"/>
       <c r="AI4" t="inlineStr">
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="AG5" s="4" t="n">
-        <v>44</v>
+        <v>210</v>
       </c>
       <c r="AH5" s="4" t="n"/>
       <c r="AI5" t="inlineStr">
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="AG6" s="4" t="n">
-        <v>63</v>
+        <v>158</v>
       </c>
       <c r="AH6" s="4" t="n"/>
       <c r="AI6" t="inlineStr">
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="AG7" s="4" t="n">
-        <v>59</v>
+        <v>163</v>
       </c>
       <c r="AH7" s="4" t="n"/>
       <c r="AI7" t="inlineStr">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="AG8" s="4" t="n">
-        <v>214</v>
+        <v>348</v>
       </c>
       <c r="AH8" s="4" t="n"/>
       <c r="AI8" t="inlineStr">
@@ -2328,7 +2328,7 @@
         </is>
       </c>
       <c r="AG9" s="4" t="n">
-        <v>47</v>
+        <v>152</v>
       </c>
       <c r="AH9" s="4" t="n"/>
       <c r="AI9" t="inlineStr">
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="AG10" s="4" t="n">
-        <v>65</v>
+        <v>166</v>
       </c>
       <c r="AH10" s="4" t="n"/>
       <c r="AI10" t="inlineStr">
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="AG11" s="4" t="n">
-        <v>43</v>
+        <v>146</v>
       </c>
       <c r="AH11" s="4" t="n"/>
       <c r="AI11" t="inlineStr">
@@ -2776,7 +2776,7 @@
         </is>
       </c>
       <c r="AG12" s="4" t="n">
-        <v>56</v>
+        <v>158</v>
       </c>
       <c r="AH12" s="4" t="n"/>
       <c r="AI12" t="inlineStr">
@@ -2924,7 +2924,7 @@
         </is>
       </c>
       <c r="AG13" s="4" t="n">
-        <v>41</v>
+        <v>175</v>
       </c>
       <c r="AH13" s="4" t="n"/>
       <c r="AI13" t="inlineStr">
@@ -3072,7 +3072,7 @@
         </is>
       </c>
       <c r="AG14" s="4" t="n">
-        <v>41</v>
+        <v>139</v>
       </c>
       <c r="AH14" s="4" t="n"/>
       <c r="AI14" t="inlineStr">
@@ -3224,7 +3224,7 @@
         </is>
       </c>
       <c r="AG15" s="4" t="n">
-        <v>59</v>
+        <v>208</v>
       </c>
       <c r="AH15" s="4" t="n"/>
       <c r="AI15" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="AG16" s="4" t="n">
-        <v>86</v>
+        <v>204</v>
       </c>
       <c r="AH16" s="4" t="n"/>
       <c r="AI16" t="inlineStr">
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="AG17" s="4" t="n">
-        <v>53</v>
+        <v>377</v>
       </c>
       <c r="AH17" s="4" t="n"/>
       <c r="AI17" t="inlineStr">
@@ -3672,7 +3672,7 @@
         </is>
       </c>
       <c r="AG18" s="4" t="n">
-        <v>210</v>
+        <v>342</v>
       </c>
       <c r="AH18" s="4" t="n"/>
       <c r="AI18" t="inlineStr">
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="AG19" s="4" t="n">
-        <v>65</v>
+        <v>189</v>
       </c>
       <c r="AH19" s="4" t="n"/>
       <c r="AI19" t="inlineStr">
@@ -3968,7 +3968,7 @@
         </is>
       </c>
       <c r="AG20" s="4" t="n">
-        <v>86</v>
+        <v>190</v>
       </c>
       <c r="AH20" s="4" t="n"/>
       <c r="AI20" t="inlineStr">
@@ -4116,7 +4116,7 @@
         </is>
       </c>
       <c r="AG21" s="4" t="n">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="AH21" s="4" t="n"/>
       <c r="AI21" t="inlineStr">
@@ -4264,7 +4264,7 @@
         </is>
       </c>
       <c r="AG22" s="4" t="n">
-        <v>12</v>
+        <v>116</v>
       </c>
       <c r="AH22" s="4" t="n"/>
       <c r="AI22" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="AG23" s="4" t="n">
-        <v>63</v>
+        <v>221</v>
       </c>
       <c r="AH23" s="4" t="n"/>
       <c r="AI23" t="inlineStr">
@@ -4560,7 +4560,7 @@
         </is>
       </c>
       <c r="AG24" s="4" t="n">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="AH24" s="4" t="n"/>
       <c r="AI24" t="inlineStr">
@@ -4708,7 +4708,7 @@
         </is>
       </c>
       <c r="AG25" s="4" t="n">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="AH25" s="4" t="n"/>
       <c r="AI25" t="inlineStr">
@@ -4860,7 +4860,7 @@
         </is>
       </c>
       <c r="AG26" s="4" t="n">
-        <v>210</v>
+        <v>354</v>
       </c>
       <c r="AH26" s="4" t="n"/>
       <c r="AI26" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="AG27" s="4" t="n">
-        <v>49</v>
+        <v>156</v>
       </c>
       <c r="AH27" s="4" t="n"/>
       <c r="AI27" t="inlineStr">
@@ -5164,7 +5164,7 @@
         </is>
       </c>
       <c r="AG28" s="4" t="n">
-        <v>59</v>
+        <v>191</v>
       </c>
       <c r="AH28" s="4" t="n"/>
       <c r="AI28" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="AG29" s="4" t="n">
-        <v>43</v>
+        <v>168</v>
       </c>
       <c r="AH29" s="4" t="n"/>
       <c r="AI29" t="inlineStr">
@@ -5460,7 +5460,7 @@
         </is>
       </c>
       <c r="AG30" s="4" t="n">
-        <v>69</v>
+        <v>164</v>
       </c>
       <c r="AH30" s="4" t="n"/>
       <c r="AI30" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="AG31" s="4" t="n">
-        <v>18</v>
+        <v>118</v>
       </c>
       <c r="AH31" s="4" t="n"/>
       <c r="AI31" t="inlineStr">
@@ -5760,7 +5760,7 @@
         </is>
       </c>
       <c r="AG32" s="4" t="n">
-        <v>33</v>
+        <v>134</v>
       </c>
       <c r="AH32" s="4" t="n"/>
       <c r="AI32" t="inlineStr">
@@ -5908,7 +5908,7 @@
         </is>
       </c>
       <c r="AG33" s="4" t="n">
-        <v>44</v>
+        <v>143</v>
       </c>
       <c r="AH33" s="4" t="n"/>
       <c r="AI33" t="inlineStr">
@@ -6056,7 +6056,7 @@
         </is>
       </c>
       <c r="AG34" s="4" t="n">
-        <v>183</v>
+        <v>314</v>
       </c>
       <c r="AH34" s="4" t="n"/>
       <c r="AI34" t="inlineStr">
@@ -6204,7 +6204,7 @@
         </is>
       </c>
       <c r="AG35" s="4" t="n">
-        <v>52</v>
+        <v>143</v>
       </c>
       <c r="AH35" s="4" t="n"/>
       <c r="AI35" t="inlineStr">
@@ -6352,7 +6352,7 @@
         </is>
       </c>
       <c r="AG36" s="4" t="n">
-        <v>91</v>
+        <v>430</v>
       </c>
       <c r="AH36" s="4" t="n"/>
       <c r="AI36" t="inlineStr">
@@ -6500,7 +6500,7 @@
         </is>
       </c>
       <c r="AG37" s="4" t="n">
-        <v>34</v>
+        <v>126</v>
       </c>
       <c r="AH37" s="4" t="n"/>
       <c r="AI37" t="inlineStr">
@@ -6648,7 +6648,7 @@
         </is>
       </c>
       <c r="AG38" s="4" t="n">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="AH38" s="4" t="n"/>
       <c r="AI38" t="inlineStr">
@@ -6796,7 +6796,7 @@
         </is>
       </c>
       <c r="AG39" s="4" t="n">
-        <v>32</v>
+        <v>127</v>
       </c>
       <c r="AH39" s="4" t="n"/>
       <c r="AI39" t="inlineStr">

</xml_diff>